<commit_message>
Chnaged numbers to percentage for KPI 6 & 7
</commit_message>
<xml_diff>
--- a/data/Program Output KPIs by $.xlsx
+++ b/data/Program Output KPIs by $.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\z003vm8n\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Learning\Miscellaneous\KPIDashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B46F50E-B8B4-4F2D-A93C-88CDCA4482E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AFD07C1-DABF-418E-B794-6CA0B30E8AF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7D6C42FC-A6F5-4FB3-BCAA-02C3B0CCB318}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{7D6C42FC-A6F5-4FB3-BCAA-02C3B0CCB318}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -107,9 +107,6 @@
     <t>Number of delivery partners trained</t>
   </si>
   <si>
-    <t>Number of delivery partners trained who are female</t>
-  </si>
-  <si>
     <t>Number of varieties released</t>
   </si>
   <si>
@@ -188,9 +185,6 @@
     <t>Number of national scientists who attended training courses</t>
   </si>
   <si>
-    <t>Number of national scientists who attended training courses who are female</t>
-  </si>
-  <si>
     <t>KPI Metric</t>
   </si>
   <si>
@@ -201,6 +195,12 @@
   </si>
   <si>
     <t>Notional Target</t>
+  </si>
+  <si>
+    <t>Percentage of delivery partners trained who are female</t>
+  </si>
+  <si>
+    <t>Percentage of national scientists who attended training courses who are female</t>
   </si>
 </sst>
 </file>
@@ -1012,10 +1012,10 @@
         <v>20</v>
       </c>
       <c r="C1" s="30" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D1" s="37" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E1" s="44">
         <v>2025</v>
@@ -1038,7 +1038,7 @@
     </row>
     <row r="2" spans="1:10" s="1" customFormat="1" ht="12.6" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="23" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B2" s="24"/>
       <c r="C2" s="25"/>
@@ -1084,7 +1084,7 @@
       </c>
       <c r="D4" s="40"/>
       <c r="E4" s="10" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F4" s="11"/>
       <c r="G4" s="11"/>
@@ -1102,7 +1102,7 @@
       </c>
       <c r="D5" s="41"/>
       <c r="E5" s="34" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F5" s="20"/>
       <c r="G5" s="20"/>
@@ -1118,7 +1118,7 @@
         <v>15</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D6" s="39">
         <v>1</v>
@@ -1136,11 +1136,11 @@
       <c r="A7" s="51"/>
       <c r="B7" s="54"/>
       <c r="C7" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D7" s="40"/>
       <c r="E7" s="10" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F7" s="11"/>
       <c r="G7" s="11"/>
@@ -1154,7 +1154,7 @@
         <v>17</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D8" s="42">
         <v>1</v>
@@ -1172,11 +1172,11 @@
       <c r="A9" s="51"/>
       <c r="B9" s="55"/>
       <c r="C9" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D9" s="42"/>
       <c r="E9" s="10" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F9" s="11"/>
       <c r="G9" s="11"/>
@@ -1208,11 +1208,11 @@
       <c r="A11" s="51"/>
       <c r="B11" s="55"/>
       <c r="C11" s="8" t="s">
-        <v>22</v>
+        <v>52</v>
       </c>
       <c r="D11" s="42"/>
       <c r="E11" s="10" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F11" s="11"/>
       <c r="G11" s="11"/>
@@ -1226,7 +1226,7 @@
         <v>19</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D12" s="42">
         <v>16</v>
@@ -1244,11 +1244,11 @@
       <c r="A13" s="52"/>
       <c r="B13" s="56"/>
       <c r="C13" s="33" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="D13" s="43"/>
       <c r="E13" s="34" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F13" s="20"/>
       <c r="G13" s="20"/>
@@ -1261,16 +1261,16 @@
         <v>3</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D14" s="39">
         <v>0.3</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F14" s="15"/>
       <c r="G14" s="15"/>
@@ -1281,14 +1281,14 @@
     <row r="15" spans="1:10" s="2" customFormat="1" ht="12" x14ac:dyDescent="0.25">
       <c r="A15" s="48"/>
       <c r="B15" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D15" s="42"/>
       <c r="E15" s="10" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F15" s="11"/>
       <c r="G15" s="11"/>
@@ -1299,14 +1299,14 @@
     <row r="16" spans="1:10" s="2" customFormat="1" ht="12" x14ac:dyDescent="0.25">
       <c r="A16" s="48"/>
       <c r="B16" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D16" s="42"/>
       <c r="E16" s="10" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F16" s="11"/>
       <c r="G16" s="11"/>
@@ -1317,7 +1317,7 @@
     <row r="17" spans="1:10" s="2" customFormat="1" ht="12" x14ac:dyDescent="0.25">
       <c r="A17" s="48"/>
       <c r="B17" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>4</v>
@@ -1337,10 +1337,10 @@
     <row r="18" spans="1:10" s="2" customFormat="1" ht="12.6" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="49"/>
       <c r="B18" s="19" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C18" s="19" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D18" s="41">
         <v>0.31</v>
@@ -1359,10 +1359,10 @@
         <v>5</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D19" s="39">
         <v>1.6</v>
@@ -1379,7 +1379,7 @@
     <row r="20" spans="1:10" s="2" customFormat="1" ht="12" x14ac:dyDescent="0.25">
       <c r="A20" s="48"/>
       <c r="B20" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>6</v>
@@ -1399,10 +1399,10 @@
     <row r="21" spans="1:10" s="2" customFormat="1" ht="12" x14ac:dyDescent="0.25">
       <c r="A21" s="48"/>
       <c r="B21" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D21" s="40">
         <v>0.13</v>
@@ -1419,10 +1419,10 @@
     <row r="22" spans="1:10" s="2" customFormat="1" ht="12" x14ac:dyDescent="0.25">
       <c r="A22" s="48"/>
       <c r="B22" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D22" s="40">
         <v>0.33</v>
@@ -1439,10 +1439,10 @@
     <row r="23" spans="1:10" s="2" customFormat="1" ht="12.6" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="49"/>
       <c r="B23" s="19" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C23" s="32" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D23" s="43">
         <v>0.22550000000000001</v>
@@ -1461,14 +1461,14 @@
         <v>7</v>
       </c>
       <c r="B24" s="13" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C24" s="13" t="s">
         <v>8</v>
       </c>
       <c r="D24" s="39"/>
       <c r="E24" s="14" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F24" s="15"/>
       <c r="G24" s="16"/>
@@ -1479,14 +1479,14 @@
     <row r="25" spans="1:10" s="2" customFormat="1" ht="12" x14ac:dyDescent="0.25">
       <c r="A25" s="48"/>
       <c r="B25" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D25" s="40"/>
       <c r="E25" s="10" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F25" s="11"/>
       <c r="G25" s="9"/>
@@ -1497,14 +1497,14 @@
     <row r="26" spans="1:10" s="2" customFormat="1" ht="12.6" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="49"/>
       <c r="B26" s="19" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C26" s="19" t="s">
         <v>10</v>
       </c>
       <c r="D26" s="41"/>
       <c r="E26" s="34" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F26" s="20"/>
       <c r="G26" s="21"/>
@@ -1514,15 +1514,15 @@
     </row>
   </sheetData>
   <mergeCells count="9">
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="B12:B13"/>
     <mergeCell ref="A24:A26"/>
     <mergeCell ref="A3:A5"/>
     <mergeCell ref="A6:A13"/>
     <mergeCell ref="A14:A18"/>
     <mergeCell ref="A19:A23"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="B12:B13"/>
   </mergeCells>
   <conditionalFormatting sqref="E3">
     <cfRule type="colorScale" priority="17">

</xml_diff>